<commit_message>
Hiding the swimmer, was annoying me too much while debugging
</commit_message>
<xml_diff>
--- a/src/server/todos.xlsx
+++ b/src/server/todos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,9 +449,20 @@
         <v>4000</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5">
+        <v>1781843360398</v>
+      </c>
+      <c r="B5" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C5">
+        <v>4000</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Commenting out the swimmer 2 to make the github build happy
</commit_message>
<xml_diff>
--- a/src/server/todos.xlsx
+++ b/src/server/todos.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -460,9 +460,31 @@
         <v>4000</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6">
+        <v>1782595680975</v>
+      </c>
+      <c r="B6" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C6">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>1782595811930</v>
+      </c>
+      <c r="B7" t="str">
+        <v>distance</v>
+      </c>
+      <c r="C7">
+        <v>4100</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>